<commit_message>
feat: add data transformation
</commit_message>
<xml_diff>
--- a/examples/sales.xlsx
+++ b/examples/sales.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\teoch\Documents\Personal\Github\approx\examples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A3039E4-963D-4E5C-936C-3757E2EF50A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89BF65BB-EA5B-49F5-9EAB-E8B3B8C6A6FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{FC993B36-9E35-4FE9-803B-9F990ACAC480}"/>
   </bookViews>
@@ -134,9 +134,6 @@
     <t>Compensation</t>
   </si>
   <si>
-    <t>Promotion Percentage</t>
-  </si>
-  <si>
     <t>S0931239E</t>
   </si>
   <si>
@@ -188,7 +185,10 @@
     <t>This is a test, very long text, goes on forever. This is not sensitive but it shall pretend to be. Can the app detect it? It keeps going on and on. No identifiable information here, maybe? But perhaps… who knows?</t>
   </si>
   <si>
-    <t>GG</t>
+    <t>Another example remark</t>
+  </si>
+  <si>
+    <t>Date of birth</t>
   </si>
 </sst>
 </file>
@@ -239,7 +239,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -579,10 +579,10 @@
   <cols>
     <col min="1" max="1" width="13.265625" customWidth="1"/>
     <col min="2" max="2" width="21.59765625" customWidth="1"/>
-    <col min="5" max="5" width="22.06640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.06640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.59765625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.46484375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.06640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.06640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.45">
@@ -596,28 +596,28 @@
         <v>6</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="J1" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="K1" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.45">
@@ -630,29 +630,29 @@
       <c r="C2">
         <v>27</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="3">
+        <v>36333</v>
+      </c>
+      <c r="E2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>14</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>19</v>
       </c>
-      <c r="G2" s="1">
+      <c r="H2" s="1">
         <v>4000</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>27</v>
       </c>
-      <c r="I2" s="1">
+      <c r="J2" s="1">
         <v>3000</v>
       </c>
-      <c r="J2" s="3">
-        <v>0.6</v>
-      </c>
       <c r="K2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.45">
@@ -665,29 +665,29 @@
       <c r="C3">
         <v>26</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="3">
+        <v>36656</v>
+      </c>
+      <c r="E3" t="s">
         <v>11</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>15</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>21</v>
       </c>
-      <c r="G3" s="1">
+      <c r="H3" s="1">
         <v>10000</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>26</v>
       </c>
-      <c r="I3" s="1">
+      <c r="J3" s="1">
         <v>7000</v>
       </c>
-      <c r="J3" s="3">
-        <v>0.2</v>
-      </c>
       <c r="K3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.45">
@@ -700,26 +700,26 @@
       <c r="C4">
         <v>66</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="3">
+        <v>22167</v>
+      </c>
+      <c r="E4" t="s">
         <v>11</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>16</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>20</v>
       </c>
-      <c r="G4" s="1">
+      <c r="H4" s="1">
         <v>30000</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>28</v>
       </c>
-      <c r="I4" s="1">
+      <c r="J4" s="1">
         <v>12000</v>
-      </c>
-      <c r="J4" s="3">
-        <v>0.05</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.45">
@@ -732,186 +732,186 @@
       <c r="C5">
         <v>45</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="3">
+        <v>29851</v>
+      </c>
+      <c r="E5" t="s">
         <v>10</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>24</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>25</v>
       </c>
-      <c r="G5" s="1">
+      <c r="H5" s="1">
         <v>50000</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>29</v>
       </c>
-      <c r="I5" s="1">
+      <c r="J5" s="1">
         <v>20000</v>
-      </c>
-      <c r="J5" s="3">
-        <v>0.1</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C6">
         <v>24</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="3">
+        <v>44718</v>
+      </c>
+      <c r="E6" t="s">
         <v>11</v>
       </c>
-      <c r="E6" t="s">
-        <v>42</v>
-      </c>
       <c r="F6" t="s">
+        <v>41</v>
+      </c>
+      <c r="G6" t="s">
         <v>21</v>
       </c>
-      <c r="G6" s="1">
+      <c r="H6" s="1">
         <v>10000</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>27</v>
       </c>
-      <c r="I6" s="1">
+      <c r="J6" s="1">
         <v>4000</v>
-      </c>
-      <c r="J6" s="3">
-        <v>0.1</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C7">
         <v>35</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="3">
+        <v>33278</v>
+      </c>
+      <c r="E7" t="s">
         <v>10</v>
       </c>
-      <c r="E7" t="s">
-        <v>43</v>
-      </c>
       <c r="F7" t="s">
+        <v>42</v>
+      </c>
+      <c r="G7" t="s">
         <v>21</v>
       </c>
-      <c r="G7" s="1">
+      <c r="H7" s="1">
         <v>20000</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>26</v>
       </c>
-      <c r="I7" s="1">
+      <c r="J7" s="1">
         <v>8000</v>
-      </c>
-      <c r="J7" s="3">
-        <v>0.2</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C8">
         <v>36</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="3">
+        <v>32880</v>
+      </c>
+      <c r="E8" t="s">
         <v>10</v>
       </c>
-      <c r="E8" t="s">
-        <v>44</v>
-      </c>
       <c r="F8" t="s">
+        <v>43</v>
+      </c>
+      <c r="G8" t="s">
         <v>21</v>
       </c>
-      <c r="G8" s="1">
+      <c r="H8" s="1">
         <v>22000</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>26</v>
       </c>
-      <c r="I8" s="1">
+      <c r="J8" s="1">
         <v>8400</v>
-      </c>
-      <c r="J8" s="3">
-        <v>0.2</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C9">
         <v>20</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="3">
+        <v>38791</v>
+      </c>
+      <c r="E9" t="s">
         <v>10</v>
       </c>
-      <c r="E9" t="s">
-        <v>45</v>
-      </c>
       <c r="F9" t="s">
+        <v>44</v>
+      </c>
+      <c r="G9" t="s">
         <v>21</v>
       </c>
-      <c r="G9" s="1">
+      <c r="H9" s="1">
         <v>12000</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>27</v>
       </c>
-      <c r="I9" s="1">
+      <c r="J9" s="1">
         <v>5000</v>
-      </c>
-      <c r="J9" s="3">
-        <v>0.25</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C10">
         <v>19</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="3">
+        <v>39312</v>
+      </c>
+      <c r="E10" t="s">
         <v>10</v>
       </c>
-      <c r="E10" t="s">
-        <v>46</v>
-      </c>
       <c r="F10" t="s">
+        <v>45</v>
+      </c>
+      <c r="G10" t="s">
         <v>21</v>
       </c>
-      <c r="G10" s="1">
+      <c r="H10" s="1">
         <v>11000</v>
       </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>27</v>
       </c>
-      <c r="I10" s="1">
+      <c r="J10" s="1">
         <v>5000</v>
-      </c>
-      <c r="J10" s="3">
-        <v>0.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>